<commit_message>
Drop trendline-direction scores to match the edited v52 sheet.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7600DC4E-848A-4EEF-A41E-5DF01FBBB6DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19300E14-3D8C-4FB0-AD58-8997BB913632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="94">
   <si>
     <t>점수 규칙 (쉬운 버전)</t>
   </si>
@@ -105,15 +105,6 @@
     <t>+1</t>
   </si>
   <si>
-    <t>추세선 방향</t>
-  </si>
-  <si>
-    <t>상승선·하락선이 둘 다 내려갈 때</t>
-  </si>
-  <si>
-    <t>둘 다 올라가지만 모이거나 평행할 때</t>
-  </si>
-  <si>
     <t>지지 근접</t>
   </si>
   <si>
@@ -299,10 +290,6 @@
   </si>
   <si>
     <t>상승 추세선에 근접 했을 때</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>둘 다 올라가는데 하락추세선이 더 크게 오를때</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
@@ -909,7 +896,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -996,10 +983,10 @@
     </row>
     <row r="8" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C8" s="5">
         <v>-1</v>
@@ -1007,10 +994,10 @@
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
@@ -1023,8 +1010,8 @@
       <c r="B10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="6">
-        <v>-1</v>
+      <c r="C10" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1032,40 +1019,40 @@
         <v>25</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" s="5">
-        <v>1</v>
+        <v>27</v>
+      </c>
+      <c r="C11" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="7">
-        <v>0</v>
+        <v>29</v>
+      </c>
+      <c r="C12" s="6">
+        <v>-2</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="5">
-        <v>1</v>
+        <v>31</v>
+      </c>
+      <c r="C13" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C14" s="7">
         <v>0</v>
@@ -1073,13 +1060,13 @@
     </row>
     <row r="15" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C15" s="6">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1087,21 +1074,21 @@
         <v>33</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" s="6">
-        <v>-1</v>
+        <v>35</v>
+      </c>
+      <c r="C16" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="7">
-        <v>0</v>
+        <v>37</v>
+      </c>
+      <c r="C17" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1109,7 +1096,7 @@
         <v>36</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C18" s="6">
         <v>-1</v>
@@ -1117,10 +1104,10 @@
     </row>
     <row r="19" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C19" s="5">
         <v>1</v>
@@ -1131,32 +1118,32 @@
         <v>39</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="5">
-        <v>1</v>
+        <v>41</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="6">
-        <v>-1</v>
+        <v>89</v>
+      </c>
+      <c r="C21" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="5">
-        <v>1</v>
+        <v>93</v>
+      </c>
+      <c r="C22" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1164,87 +1151,87 @@
         <v>42</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C23" s="6">
-        <v>0</v>
+        <v>85</v>
+      </c>
+      <c r="C23" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C24" s="7">
-        <v>0</v>
+        <v>86</v>
+      </c>
+      <c r="C24" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="4" t="s">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C25" s="7">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C26" s="5">
+        <v>91</v>
+      </c>
+      <c r="C26" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C27" s="6">
+        <v>92</v>
+      </c>
+      <c r="C27" s="7">
         <v>-1</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C28" s="7">
-        <v>0</v>
+        <v>44</v>
+      </c>
+      <c r="C28" s="6">
+        <v>-2</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>94</v>
+        <v>43</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="C29" s="6">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>94</v>
+        <v>46</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C30" s="7">
-        <v>-1</v>
+        <v>47</v>
+      </c>
+      <c r="C30" s="5">
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1252,21 +1239,21 @@
         <v>46</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C31" s="6">
-        <v>-2</v>
+        <v>48</v>
+      </c>
+      <c r="C31" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C32" s="6">
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1274,10 +1261,10 @@
         <v>49</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" s="5">
-        <v>2</v>
+        <v>51</v>
+      </c>
+      <c r="C33" s="6">
+        <v>-2</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1285,58 +1272,25 @@
         <v>49</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C34" s="5">
-        <v>1</v>
+        <v>52</v>
+      </c>
+      <c r="C34" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C35" s="6">
-        <v>-3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C36" s="6">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C37" s="6">
         <v>-1</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C38" s="6">
-        <v>-1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C38" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C35" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1365,10 +1319,10 @@
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C2" s="7">
         <v>0</v>
@@ -1376,10 +1330,10 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C3" s="6">
         <v>-1</v>
@@ -1387,10 +1341,10 @@
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>24</v>
@@ -1398,10 +1352,10 @@
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C5" s="7">
         <v>0</v>
@@ -1409,10 +1363,10 @@
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C6" s="6">
         <v>-1</v>
@@ -1420,10 +1374,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
@@ -1431,7 +1385,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1457,77 +1411,77 @@
   <sheetData>
     <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="9" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="13" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" s="18" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B10" s="17"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11" s="18" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B11" s="17"/>
     </row>

</xml_diff>

<commit_message>
Score -1 when price fully breaks below the uptrend line.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19300E14-3D8C-4FB0-AD58-8997BB913632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44793A6D-0C00-418C-98F2-9E96BD34EB26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="95">
   <si>
     <t>점수 규칙 (쉬운 버전)</t>
   </si>
@@ -325,6 +325,10 @@
   </si>
   <si>
     <t>현재가가 비싼 구간 인데 횡보하거나 하락 추세일때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>현재가가 상승 추세선을 완전 이탈했을 때</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -896,7 +900,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1005,13 +1009,13 @@
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="5">
-        <v>1</v>
+        <v>94</v>
+      </c>
+      <c r="C10" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1019,32 +1023,32 @@
         <v>25</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="7">
-        <v>0</v>
+        <v>26</v>
+      </c>
+      <c r="C11" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="6">
-        <v>-2</v>
+        <v>27</v>
+      </c>
+      <c r="C12" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C13" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1052,21 +1056,21 @@
         <v>30</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="7">
-        <v>0</v>
+        <v>31</v>
+      </c>
+      <c r="C14" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="6">
-        <v>-1</v>
+        <v>32</v>
+      </c>
+      <c r="C15" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1074,18 +1078,18 @@
         <v>33</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="5">
-        <v>1</v>
+        <v>34</v>
+      </c>
+      <c r="C16" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C17" s="5">
         <v>1</v>
@@ -1096,21 +1100,21 @@
         <v>36</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="6">
-        <v>-1</v>
+        <v>37</v>
+      </c>
+      <c r="C18" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C19" s="5">
-        <v>1</v>
+        <v>38</v>
+      </c>
+      <c r="C19" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1118,20 +1122,20 @@
         <v>39</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="6">
-        <v>0</v>
+        <v>40</v>
+      </c>
+      <c r="C20" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C21" s="7">
+        <v>41</v>
+      </c>
+      <c r="C21" s="6">
         <v>0</v>
       </c>
     </row>
@@ -1140,21 +1144,21 @@
         <v>88</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C22" s="7">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C23" s="5">
-        <v>1</v>
+        <v>93</v>
+      </c>
+      <c r="C23" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1162,10 +1166,10 @@
         <v>42</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C24" s="6">
-        <v>-1</v>
+        <v>85</v>
+      </c>
+      <c r="C24" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1173,21 +1177,21 @@
         <v>42</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C25" s="7">
-        <v>0</v>
+        <v>86</v>
+      </c>
+      <c r="C25" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C26" s="6">
-        <v>1</v>
+        <v>87</v>
+      </c>
+      <c r="C26" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1195,21 +1199,21 @@
         <v>90</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C27" s="7">
-        <v>-1</v>
+        <v>91</v>
+      </c>
+      <c r="C27" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C28" s="6">
-        <v>-2</v>
+        <v>92</v>
+      </c>
+      <c r="C28" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1217,21 +1221,21 @@
         <v>43</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C29" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C30" s="5">
-        <v>2</v>
+        <v>45</v>
+      </c>
+      <c r="C30" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1239,21 +1243,21 @@
         <v>46</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C31" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C32" s="6">
-        <v>-3</v>
+        <v>48</v>
+      </c>
+      <c r="C32" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1261,10 +1265,10 @@
         <v>49</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C33" s="6">
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1272,25 +1276,36 @@
         <v>49</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C34" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C35" s="6">
         <v>-1</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C36" s="6">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C35" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C36" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
VAH above is always -1; tighten 6-month gain penalties.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44793A6D-0C00-418C-98F2-9E96BD34EB26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FB04A55-FFF1-473A-91B1-8799CC852B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="96">
   <si>
     <t>점수 규칙 (쉬운 버전)</t>
   </si>
@@ -308,10 +308,6 @@
     <t>밸류 상단 (VAH)</t>
   </si>
   <si>
-    <t>현재가가 비싼 구간 위여도 상승 추세일때</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>20일선</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -324,11 +320,19 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>현재가가 비싼 구간 인데 횡보하거나 하락 추세일때</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>현재가가 상승 추세선을 완전 이탈했을 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>현재가가 비싼 구간 위</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>현재가가 비싼 구간 인데</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 동안 50% 이상 100% 미만 오름</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -900,7 +904,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1012,7 +1016,7 @@
         <v>83</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C10" s="7">
         <v>-1</v>
@@ -1144,10 +1148,10 @@
         <v>88</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C22" s="7">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1155,7 +1159,7 @@
         <v>88</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C23" s="7">
         <v>-1</v>
@@ -1196,10 +1200,10 @@
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>91</v>
       </c>
       <c r="C27" s="6">
         <v>1</v>
@@ -1207,10 +1211,10 @@
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C28" s="7">
         <v>-1</v>
@@ -1268,7 +1272,7 @@
         <v>50</v>
       </c>
       <c r="C33" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1279,7 +1283,7 @@
         <v>51</v>
       </c>
       <c r="C34" s="6">
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1290,22 +1294,33 @@
         <v>52</v>
       </c>
       <c r="C35" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="C36" s="6">
         <v>-1</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C37" s="6">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C36" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C37" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Raise sell cuts to 45/40/30 to match the edited sheet.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FB04A55-FFF1-473A-91B1-8799CC852B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76011E9-0597-4830-9AD7-63A7E7B7F5DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="이렇게 봐요" sheetId="1" r:id="rId1"/>
@@ -261,18 +261,6 @@
     <t>가까운 가격: 하루 변동폭의 약 절반, 또는 주가의 0.8% 중 더 큰 값.</t>
   </si>
   <si>
-    <t>40% 초과 ~ 70% 미만</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>35% 초과 ~ 40% 이하</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>30% 초과 ~ 35% 이하</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>30% 이하</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -333,6 +321,18 @@
   </si>
   <si>
     <t>6개월 동안 50% 이상 100% 미만 오름</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>40% 초과 ~ 45% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>30% 초과 ~ 40% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>45% 초과 ~ 70% 미만</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -991,10 +991,10 @@
     </row>
     <row r="8" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C8" s="5">
         <v>-1</v>
@@ -1002,10 +1002,10 @@
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
@@ -1013,10 +1013,10 @@
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C10" s="7">
         <v>-1</v>
@@ -1145,10 +1145,10 @@
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C22" s="7">
         <v>-1</v>
@@ -1156,10 +1156,10 @@
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C23" s="7">
         <v>-1</v>
@@ -1170,7 +1170,7 @@
         <v>42</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C24" s="5">
         <v>1</v>
@@ -1181,7 +1181,7 @@
         <v>42</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C25" s="6">
         <v>-1</v>
@@ -1192,7 +1192,7 @@
         <v>42</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C26" s="7">
         <v>0</v>
@@ -1200,10 +1200,10 @@
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C27" s="6">
         <v>1</v>
@@ -1211,10 +1211,10 @@
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C28" s="7">
         <v>-1</v>
@@ -1302,7 +1302,7 @@
         <v>49</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C36" s="6">
         <v>-1</v>
@@ -1473,7 +1473,7 @@
     </row>
     <row r="5" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="11" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>71</v>
@@ -1481,7 +1481,7 @@
     </row>
     <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="13" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>72</v>
@@ -1489,7 +1489,7 @@
     </row>
     <row r="7" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>73</v>
@@ -1497,7 +1497,7 @@
     </row>
     <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="14" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>74</v>

</xml_diff>

<commit_message>
Score -1 when both trendlines slope down, matching the sheet.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76011E9-0597-4830-9AD7-63A7E7B7F5DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{926E24C1-919D-467A-9C57-C73A26B9973C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="이렇게 봐요" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="98">
   <si>
     <t>점수 규칙 (쉬운 버전)</t>
   </si>
@@ -333,6 +333,14 @@
   </si>
   <si>
     <t>45% 초과 ~ 70% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>추세선 방향</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>하락 추세선 상승 추세선 모두 하락일 때</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -904,7 +912,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1002,13 +1010,13 @@
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" s="7">
-        <v>1</v>
+        <v>97</v>
+      </c>
+      <c r="C9" s="5">
+        <v>-1</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1016,21 +1024,21 @@
         <v>80</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C10" s="7">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="5">
-        <v>1</v>
+        <v>89</v>
+      </c>
+      <c r="C11" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1038,32 +1046,32 @@
         <v>25</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="7">
-        <v>0</v>
+        <v>26</v>
+      </c>
+      <c r="C12" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="6">
-        <v>-2</v>
+        <v>27</v>
+      </c>
+      <c r="C13" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C14" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1071,21 +1079,21 @@
         <v>30</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="7">
-        <v>0</v>
+        <v>31</v>
+      </c>
+      <c r="C15" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" s="6">
-        <v>-1</v>
+        <v>32</v>
+      </c>
+      <c r="C16" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1093,18 +1101,18 @@
         <v>33</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="5">
-        <v>1</v>
+        <v>34</v>
+      </c>
+      <c r="C17" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C18" s="5">
         <v>1</v>
@@ -1115,21 +1123,21 @@
         <v>36</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C19" s="6">
-        <v>-1</v>
+        <v>37</v>
+      </c>
+      <c r="C19" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="5">
-        <v>1</v>
+        <v>38</v>
+      </c>
+      <c r="C20" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1137,21 +1145,21 @@
         <v>39</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="6">
-        <v>0</v>
+        <v>40</v>
+      </c>
+      <c r="C21" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C22" s="7">
-        <v>-1</v>
+        <v>41</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1159,7 +1167,7 @@
         <v>85</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C23" s="7">
         <v>-1</v>
@@ -1167,13 +1175,13 @@
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C24" s="5">
-        <v>1</v>
+        <v>91</v>
+      </c>
+      <c r="C24" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1181,10 +1189,10 @@
         <v>42</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C25" s="6">
-        <v>-1</v>
+        <v>82</v>
+      </c>
+      <c r="C25" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1192,21 +1200,21 @@
         <v>42</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C26" s="7">
-        <v>0</v>
+        <v>83</v>
+      </c>
+      <c r="C26" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C27" s="6">
-        <v>1</v>
+        <v>84</v>
+      </c>
+      <c r="C27" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1214,21 +1222,21 @@
         <v>86</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C28" s="7">
-        <v>-1</v>
+        <v>87</v>
+      </c>
+      <c r="C28" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>43</v>
+        <v>86</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C29" s="6">
-        <v>-2</v>
+        <v>88</v>
+      </c>
+      <c r="C29" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1236,21 +1244,21 @@
         <v>43</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C30" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C31" s="5">
-        <v>2</v>
+        <v>45</v>
+      </c>
+      <c r="C31" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1258,21 +1266,21 @@
         <v>46</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C32" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" s="6">
-        <v>-4</v>
+        <v>48</v>
+      </c>
+      <c r="C33" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1280,10 +1288,10 @@
         <v>49</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C34" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1291,10 +1299,10 @@
         <v>49</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C35" s="6">
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1302,25 +1310,36 @@
         <v>49</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="C36" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C37" s="6">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B38" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C37" s="6">
+      <c r="C38" s="6">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C37" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C38" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Split buy/sell cuts into stock and crypto tables.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{926E24C1-919D-467A-9C57-C73A26B9973C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59834593-6FFC-47ED-BBA7-3F1F914BE320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="이렇게 봐요" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,8 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$2:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="109">
   <si>
     <t>점수 규칙 (쉬운 버전)</t>
   </si>
@@ -341,6 +341,50 @@
   </si>
   <si>
     <t>하락 추세선 상승 추세선 모두 하락일 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>코인</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>주식</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>65% 이상 ~ 70% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>70% 이상 ~ 75% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>75% 이상</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>35% 초과 ~ 70% 미만</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>30% 초과 ~ 35% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>25% 초과 ~ 30% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>25% 이하</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>1년 장기 상승추세</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">1년 동안 </t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -446,7 +490,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -469,11 +513,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -523,6 +576,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -912,7 +968,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1329,17 +1385,26 @@
     </row>
     <row r="38" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C38" s="6"/>
+    </row>
+    <row r="39" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A39" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B39" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C38" s="6">
+      <c r="C39" s="6">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C38" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C39" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1451,94 +1516,166 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A1" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="D1" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="E1" s="19"/>
+    </row>
+    <row r="2" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="8" t="s">
+      <c r="D2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B3" s="5" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="8" t="s">
+      <c r="D3" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B4" s="5" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="9" t="s">
+      <c r="D4" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B5" s="10" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="11" t="s">
+      <c r="D5" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B6" s="12" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="13" t="s">
+      <c r="D6" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B7" s="6" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="13" t="s">
+      <c r="D7" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B8" s="6" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="14" t="s">
+      <c r="D8" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B9" s="15" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A10" s="18" t="s">
+      <c r="D9" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="B10" s="17"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A11" s="18" t="s">
+      <c r="B11" s="17"/>
+      <c r="D11" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="17"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A12" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="D12" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" s="17"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <mergeCells count="2">
+  <autoFilter ref="A2:B9" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <mergeCells count="6">
+    <mergeCell ref="A12:B12"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Simplify 6-month gain penalties to 50% and 100% only.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59834593-6FFC-47ED-BBA7-3F1F914BE320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794B49D8-8FFE-4294-85A7-4D95300DB19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="이렇게 봐요" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$2:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="105">
   <si>
     <t>점수 규칙 (쉬운 버전)</t>
   </si>
@@ -180,15 +180,6 @@
     <t>6개월 상승률</t>
   </si>
   <si>
-    <t>6개월 동안 400% 이상 오름</t>
-  </si>
-  <si>
-    <t>6개월 동안 300% 이상 400% 미만 오름</t>
-  </si>
-  <si>
-    <t>6개월 동안 100% 이상 300% 미만 오름</t>
-  </si>
-  <si>
     <t>손익비</t>
   </si>
   <si>
@@ -380,11 +371,7 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>1년 장기 상승추세</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">1년 동안 </t>
+    <t>6개월 동안 100% 이상오름</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -968,7 +955,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1055,10 +1042,10 @@
     </row>
     <row r="8" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C8" s="5">
         <v>-1</v>
@@ -1066,10 +1053,10 @@
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C9" s="5">
         <v>-1</v>
@@ -1077,10 +1064,10 @@
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
@@ -1088,10 +1075,10 @@
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C11" s="7">
         <v>-1</v>
@@ -1220,10 +1207,10 @@
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C23" s="7">
         <v>-1</v>
@@ -1231,10 +1218,10 @@
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C24" s="7">
         <v>-1</v>
@@ -1245,7 +1232,7 @@
         <v>42</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C25" s="5">
         <v>1</v>
@@ -1256,7 +1243,7 @@
         <v>42</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C26" s="6">
         <v>-1</v>
@@ -1267,7 +1254,7 @@
         <v>42</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C27" s="7">
         <v>0</v>
@@ -1275,10 +1262,10 @@
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C28" s="6">
         <v>1</v>
@@ -1286,10 +1273,10 @@
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C29" s="7">
         <v>-1</v>
@@ -1344,10 +1331,10 @@
         <v>49</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="C34" s="6">
-        <v>-4</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1355,56 +1342,25 @@
         <v>49</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="C35" s="6">
-        <v>-3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C36" s="6">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C37" s="6">
         <v>-1</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="C38" s="6"/>
-    </row>
-    <row r="39" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C39" s="6">
-        <v>-1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C39" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C36" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1433,10 +1389,10 @@
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C2" s="7">
         <v>0</v>
@@ -1444,10 +1400,10 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C3" s="6">
         <v>-1</v>
@@ -1455,10 +1411,10 @@
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>58</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>24</v>
@@ -1466,10 +1422,10 @@
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C5" s="7">
         <v>0</v>
@@ -1477,10 +1433,10 @@
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C6" s="6">
         <v>-1</v>
@@ -1488,10 +1444,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
@@ -1499,7 +1455,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1527,143 +1483,143 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B1" s="19"/>
       <c r="D1" s="19" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E1" s="19"/>
     </row>
     <row r="2" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="13" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="18" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B11" s="17"/>
       <c r="D11" s="18" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E11" s="17"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="18" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B12" s="17"/>
       <c r="D12" s="18" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E12" s="17"/>
     </row>

</xml_diff>

<commit_message>
Add 1-month uptrend bonus on long lookbacks and MA200 near score.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794B49D8-8FFE-4294-85A7-4D95300DB19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F063FBC-DD93-4929-B3F3-934CC6B3E870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$2:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="108">
   <si>
     <t>점수 규칙 (쉬운 버전)</t>
   </si>
@@ -372,6 +372,18 @@
   </si>
   <si>
     <t>6개월 동안 100% 이상오름</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>200일선</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>현재가가 200일선 아래위로 근처일 때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>조회 기간이 3개월 이상이고, 조회기간 1개월 조회시 상승 추세일때</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -955,7 +967,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1034,29 +1046,29 @@
         <v>18</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="7">
-        <v>0</v>
+        <v>107</v>
+      </c>
+      <c r="C7" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C8" s="5">
-        <v>-1</v>
+        <v>23</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="C9" s="5">
         <v>-1</v>
@@ -1064,13 +1076,13 @@
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="7">
-        <v>1</v>
+        <v>94</v>
+      </c>
+      <c r="C10" s="5">
+        <v>-1</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1078,21 +1090,21 @@
         <v>77</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C11" s="7">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>25</v>
+        <v>77</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="5">
-        <v>1</v>
+        <v>86</v>
+      </c>
+      <c r="C12" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1100,32 +1112,32 @@
         <v>25</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="7">
-        <v>0</v>
+        <v>26</v>
+      </c>
+      <c r="C13" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="6">
-        <v>-2</v>
+        <v>27</v>
+      </c>
+      <c r="C14" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C15" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1133,21 +1145,21 @@
         <v>30</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="7">
-        <v>0</v>
+        <v>31</v>
+      </c>
+      <c r="C16" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="6">
-        <v>-1</v>
+        <v>32</v>
+      </c>
+      <c r="C17" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1155,18 +1167,18 @@
         <v>33</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" s="5">
-        <v>1</v>
+        <v>34</v>
+      </c>
+      <c r="C18" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C19" s="5">
         <v>1</v>
@@ -1177,21 +1189,21 @@
         <v>36</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="6">
-        <v>-1</v>
+        <v>37</v>
+      </c>
+      <c r="C20" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21" s="5">
-        <v>1</v>
+        <v>38</v>
+      </c>
+      <c r="C21" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1199,21 +1211,21 @@
         <v>39</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" s="6">
-        <v>0</v>
+        <v>40</v>
+      </c>
+      <c r="C22" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C23" s="7">
-        <v>-1</v>
+        <v>41</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1221,7 +1233,7 @@
         <v>82</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C24" s="7">
         <v>-1</v>
@@ -1229,13 +1241,13 @@
     </row>
     <row r="25" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="4" t="s">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C25" s="5">
-        <v>1</v>
+        <v>88</v>
+      </c>
+      <c r="C25" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1243,10 +1255,10 @@
         <v>42</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C26" s="6">
-        <v>-1</v>
+        <v>79</v>
+      </c>
+      <c r="C26" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1254,21 +1266,21 @@
         <v>42</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C27" s="7">
-        <v>0</v>
+        <v>80</v>
+      </c>
+      <c r="C27" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>83</v>
+        <v>42</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C28" s="6">
-        <v>1</v>
+        <v>81</v>
+      </c>
+      <c r="C28" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1276,91 +1288,113 @@
         <v>83</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C29" s="7">
-        <v>-1</v>
+        <v>84</v>
+      </c>
+      <c r="C29" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>43</v>
+        <v>83</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C30" s="6">
-        <v>-2</v>
+        <v>85</v>
+      </c>
+      <c r="C30" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="4" t="s">
-        <v>43</v>
+        <v>105</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C31" s="6">
-        <v>-1</v>
+        <v>106</v>
+      </c>
+      <c r="C31" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C32" s="5">
-        <v>2</v>
+        <v>44</v>
+      </c>
+      <c r="C32" s="6">
+        <v>-2</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C33" s="5">
-        <v>1</v>
+        <v>45</v>
+      </c>
+      <c r="C33" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C34" s="6">
-        <v>-2</v>
+        <v>47</v>
+      </c>
+      <c r="C34" s="5">
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C35" s="6">
-        <v>-1</v>
+        <v>48</v>
+      </c>
+      <c r="C35" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C36" s="6">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" s="6">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B38" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C36" s="6">
+      <c r="C38" s="6">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C36" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C38" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Drop weak-volume upside bonus; flatten 1-month gain and loss scores.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F063FBC-DD93-4929-B3F3-934CC6B3E870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0287EE86-B93B-4971-86E3-D6AF0F8F593D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$2:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="105">
   <si>
     <t>점수 규칙 (쉬운 버전)</t>
   </si>
@@ -135,9 +135,6 @@
     <t>아래 지지 매물대가 약하고, 그 아래 다음 지지가 10% 이상 떨어져 있을 때</t>
   </si>
   <si>
-    <t>아래 지지 매물대가 약하고, 위 저항이 10% 이상 떨어져 있을 때</t>
-  </si>
-  <si>
     <t>최대 매물 (POC)</t>
   </si>
   <si>
@@ -162,21 +159,9 @@
     <t>1개월 상승률</t>
   </si>
   <si>
-    <t>한 달 동안 100% 이상 오름</t>
-  </si>
-  <si>
-    <t>한 달 동안 30% 이상 100% 미만 오름</t>
-  </si>
-  <si>
     <t>1개월 하락률</t>
   </si>
   <si>
-    <t>한 달 동안 30% 이상 떨어짐</t>
-  </si>
-  <si>
-    <t>한 달 동안 20% 이상 30% 미만 떨어짐</t>
-  </si>
-  <si>
     <t>6개월 상승률</t>
   </si>
   <si>
@@ -375,15 +360,23 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>200일선</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>현재가가 200일선 아래위로 근처일 때</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
     <t>조회 기간이 3개월 이상이고, 조회기간 1개월 조회시 상승 추세일때</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달 동안 30% 이상 오름</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>180일선</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>한 달 동안 20% 이상 떨어짐</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -967,7 +960,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1046,7 +1039,7 @@
         <v>18</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C7" s="6">
         <v>1</v>
@@ -1065,10 +1058,10 @@
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C9" s="5">
         <v>-1</v>
@@ -1076,10 +1069,10 @@
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C10" s="5">
         <v>-1</v>
@@ -1087,10 +1080,10 @@
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C11" s="7">
         <v>1</v>
@@ -1098,10 +1091,10 @@
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C12" s="7">
         <v>-1</v>
@@ -1175,10 +1168,10 @@
     </row>
     <row r="19" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C19" s="5">
         <v>1</v>
@@ -1186,54 +1179,54 @@
     </row>
     <row r="20" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="5">
-        <v>1</v>
+      <c r="C20" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" s="6">
-        <v>-1</v>
+        <v>39</v>
+      </c>
+      <c r="C21" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="5">
-        <v>1</v>
+      <c r="C22" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="6">
-        <v>0</v>
+        <v>82</v>
+      </c>
+      <c r="C23" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C24" s="7">
         <v>-1</v>
@@ -1241,79 +1234,79 @@
     </row>
     <row r="25" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="4" t="s">
-        <v>82</v>
+        <v>41</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C25" s="7">
-        <v>-1</v>
+        <v>74</v>
+      </c>
+      <c r="C25" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C26" s="5">
-        <v>1</v>
+        <v>75</v>
+      </c>
+      <c r="C26" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C27" s="6">
-        <v>-1</v>
+        <v>76</v>
+      </c>
+      <c r="C27" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C28" s="7">
-        <v>0</v>
+        <v>79</v>
+      </c>
+      <c r="C28" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C29" s="6">
-        <v>1</v>
+        <v>80</v>
+      </c>
+      <c r="C29" s="7">
+        <v>-1</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="C30" s="7">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="4" t="s">
-        <v>105</v>
+        <v>42</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C31" s="7">
-        <v>1</v>
+        <v>102</v>
+      </c>
+      <c r="C31" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1321,80 +1314,47 @@
         <v>43</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C32" s="6">
-        <v>-2</v>
+        <v>104</v>
+      </c>
+      <c r="C32" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>45</v>
+        <v>99</v>
       </c>
       <c r="C33" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="5">
-        <v>2</v>
+        <v>84</v>
+      </c>
+      <c r="C34" s="6">
+        <v>-1</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C35" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C36" s="6">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C37" s="6">
+      <c r="C35" s="6">
         <v>-1</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C38" s="6">
-        <v>-1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C38" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C35" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1423,10 +1383,10 @@
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C2" s="7">
         <v>0</v>
@@ -1434,10 +1394,10 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C3" s="6">
         <v>-1</v>
@@ -1445,10 +1405,10 @@
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>24</v>
@@ -1456,10 +1416,10 @@
     </row>
     <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C5" s="7">
         <v>0</v>
@@ -1467,10 +1427,10 @@
     </row>
     <row r="6" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>57</v>
       </c>
       <c r="C6" s="6">
         <v>-1</v>
@@ -1478,10 +1438,10 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
@@ -1489,7 +1449,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1517,143 +1477,143 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B1" s="19"/>
       <c r="D1" s="19" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E1" s="19"/>
     </row>
     <row r="2" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="9" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="13" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="14" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="18" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B11" s="17"/>
       <c r="D11" s="18" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E11" s="17"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="18" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B12" s="17"/>
       <c r="D12" s="18" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E12" s="17"/>
     </row>

</xml_diff>

<commit_message>
Add a -3 penalty when 6-month return is 600% or more.
Live scoring now uses 600%/-3, 100%/-2, 50%/-1 as mutually exclusive tiers.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0287EE86-B93B-4971-86E3-D6AF0F8F593D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36E8B9FA-55D3-4CE6-AE53-0A1243A9F109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="매수 매도 기준" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'매수 매도 기준'!$A$2:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="106">
   <si>
     <t>점수 규칙 (쉬운 버전)</t>
   </si>
@@ -296,10 +296,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>6개월 동안 50% 이상 100% 미만 오름</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>40% 초과 ~ 45% 이하</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -356,14 +352,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>6개월 동안 100% 이상오름</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>현재가가 200일선 아래위로 근처일 때</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>조회 기간이 3개월 이상이고, 조회기간 1개월 조회시 상승 추세일때</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -377,6 +365,23 @@
   </si>
   <si>
     <t>한 달 동안 20% 이상 떨어짐</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>현재가가 180일선 아래위로 근처일 때(6개월 수익률용으로 일봉을 220일까지 받고
+• 주말·휴장이면 다음 거래일 종가로 계산합니다.)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 동안 800% 이상오름</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 동안 50% 이상 200% 미만 오름</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>6개월 동안 200% 이상오름 800%미만오름</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -960,7 +965,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1039,7 +1044,7 @@
         <v>18</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C7" s="6">
         <v>1</v>
@@ -1069,10 +1074,10 @@
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="C10" s="5">
         <v>-1</v>
@@ -1289,10 +1294,10 @@
     </row>
     <row r="30" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C30" s="7">
         <v>1</v>
@@ -1303,7 +1308,7 @@
         <v>42</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C31" s="6">
         <v>-1</v>
@@ -1314,7 +1319,7 @@
         <v>43</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C32" s="5">
         <v>1</v>
@@ -1325,10 +1330,10 @@
         <v>44</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C33" s="6">
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
@@ -1336,25 +1341,36 @@
         <v>44</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="C34" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>46</v>
+        <v>104</v>
       </c>
       <c r="C35" s="6">
         <v>-1</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C36" s="6">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C35" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C36" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1477,11 +1493,11 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B1" s="19"/>
       <c r="D1" s="19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E1" s="19"/>
     </row>
@@ -1507,7 +1523,7 @@
         <v>58</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>58</v>
@@ -1521,7 +1537,7 @@
         <v>60</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>60</v>
@@ -1535,7 +1551,7 @@
         <v>62</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>62</v>
@@ -1543,13 +1559,13 @@
     </row>
     <row r="6" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>63</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>63</v>
@@ -1557,13 +1573,13 @@
     </row>
     <row r="7" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>64</v>
@@ -1571,13 +1587,13 @@
     </row>
     <row r="8" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>65</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>65</v>
@@ -1591,7 +1607,7 @@
         <v>66</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>66</v>

</xml_diff>

<commit_message>
Add a +1 bonus when the 2-month window is up on 3-month+ lookbacks.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="매수 매도 기준" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v68</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v69</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -792,37 +792,39 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>횡보일 때</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>0</v>
+          <t>조회 기간이 3개월 이상이고, 조회기간 2개월 조회시 상승 추세일때</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>하락 추세선 근접</t>
+          <t>추세</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>하락 추세선에 근접 했을 때</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>-1</v>
+          <t>횡보일 때</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>추세선 방향</t>
+          <t>하락 추세선 근접</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>하락 추세선 상승 추세선 모두 하락일 때</t>
+          <t>하락 추세선에 근접 했을 때</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
@@ -832,18 +834,16 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>상승 추세선 근접</t>
+          <t>추세선 방향</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>상승 추세선에 근접 했을 때</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>하락 추세선 상승 추세선 모두 하락일 때</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
@@ -854,28 +854,28 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>현재가가 상승 추세선을 완전 이탈했을 때, 이탈후 최근봉 4봉이 지났으면 무효</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>-1</v>
+          <t>상승 추세선에 근접 했을 때</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>지지 근접</t>
+          <t>상승 추세선 근접</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>지지선 바로 옆이고, 강도 4 이상일 때</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>현재가가 상승 추세선을 완전 이탈했을 때, 이탈후 최근봉 4봉이 지났으면 무효</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
@@ -886,41 +886,43 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>지지선 바로 옆이지만 강도가 4보다 약할 때</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>0</v>
+          <t>지지선 바로 옆이고, 강도 4 이상일 때</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>지지 이탈</t>
+          <t>지지 근접</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>현재가가 지지선보다 뚜렷이 아래일 때</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>-2</v>
+          <t>지지선 바로 옆이지만 강도가 4보다 약할 때</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>저항 근접</t>
+          <t>지지 이탈</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>저항선 바로 옆이고, 강도 4 이상일 때</t>
+          <t>현재가가 지지선보다 뚜렷이 아래일 때</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
@@ -931,43 +933,41 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>저항선 바로 옆이지만 강도가 4보다 약할 때</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>0</v>
+          <t>저항선 바로 옆이고, 강도 4 이상일 때</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>약한 매물대</t>
+          <t>저항 근접</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>아래 지지 매물대가 약하고, 그 아래 다음 지지가 10% 이상 떨어져 있을 때</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>-1</v>
+          <t>저항선 바로 옆이지만 강도가 4보다 약할 때</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>최대 매물 (POC)</t>
+          <t>약한 매물대</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>현재가가 거래가 가장 많았던 가격 근처이고, 상승 추세</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>아래 지지 매물대가 약하고, 그 아래 다음 지지가 10% 이상 떨어져 있을 때</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
@@ -978,28 +978,28 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>현재가가 그 가격 근처이고, 하락 추세</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>-1</v>
+          <t>현재가가 거래가 가장 많았던 가격 근처이고, 상승 추세</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>밸류 하단 (VAL)</t>
+          <t>최대 매물 (POC)</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>현재가가 싼 구간 아래이고, 상승 추세</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>현재가가 그 가격 근처이고, 하락 추세</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
@@ -1010,43 +1010,43 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>현재가가 싼 구간 아래이고, 하락 추세</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n">
-        <v>0</v>
+          <t>현재가가 싼 구간 아래이고, 상승 추세</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>밸류 상단 (VAH)</t>
+          <t>밸류 하단 (VAL)</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>현재가가 비싼 구간 위</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="n">
-        <v>-1</v>
+          <t>현재가가 싼 구간 아래이고, 하락 추세</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>밸류 상단 (VAH)</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>30 이하 (너무 많이 떨어짐)</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>현재가가 비싼 구간 위</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="25" ht="32" customHeight="1">
@@ -1057,11 +1057,13 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>70 이상 (너무 많이 오름)</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="n">
-        <v>-1</v>
+          <t>30 이하 (너무 많이 떨어짐)</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="32" customHeight="1">
@@ -1072,28 +1074,26 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>30~70 사이</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="n">
-        <v>0</v>
+          <t>70 이상 (너무 많이 오름)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>20일선</t>
+          <t>RSI</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>현재가가 20일선보다 아래이고, 상승 추세일때</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>30~70 사이</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28" ht="32" customHeight="1">
@@ -1104,11 +1104,13 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>현재가가 20일선보다 아래이고, 하락 추세일때</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>-1</v>
+          <t>현재가가 20일선보다 아래이고, 상승 추세일때</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1">
@@ -1119,39 +1121,37 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>현재가가 20일선보다 아래이고, 횡보일 때</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="n">
-        <v>0</v>
+          <t>현재가가 20일선보다 아래이고, 하락 추세일때</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>60일선</t>
+          <t>20일선</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>현재가가 60일(봉)선 근처일 때</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>현재가가 20일선보다 아래이고, 횡보일 때</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="32" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>180일선</t>
+          <t>60일선</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>현재가가 장기 이평 근처일 때. 6개월 조회는 180일선, 1년 조회는 200일선</t>
+          <t>현재가가 60일(봉)선 근처일 때</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -1163,33 +1163,33 @@
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>1개월 상승률</t>
+          <t>180일선</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 30% 이상 오름</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="n">
-        <v>-1</v>
+          <t>현재가가 장기 이평 근처일 때. 6개월 조회는 180일선, 1년 조회는 200일선</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>1개월 하락률</t>
+          <t>1개월 상승률</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 1%이상 20%미만 하락했을시</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>한 달 동안 30% 이상 오름</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="34" ht="32" customHeight="1">
@@ -1200,12 +1200,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 20% 이상 떨어짐</t>
+          <t>한 달 동안 1%이상 20%미만 하락했을시</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+1</t>
         </is>
       </c>
     </row>
@@ -1217,28 +1217,30 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 40% 이상 떨어짐</t>
+          <t>한 달 동안 20% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+2</t>
         </is>
       </c>
     </row>
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>6개월 상승률</t>
+          <t>1개월 하락률</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 800% 이상 오름</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="n">
-        <v>-3</v>
+          <t>한 달 동안 40% 이상 떨어짐</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>+3</t>
+        </is>
       </c>
     </row>
     <row r="37" ht="32" customHeight="1">
@@ -1249,11 +1251,11 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 200% 이상 800% 미만 오름</t>
+          <t>6개월 동안 800% 이상 오름</t>
         </is>
       </c>
       <c r="C37" s="7" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="38" ht="32" customHeight="1">
@@ -1264,30 +1266,45 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 50% 이상 200% 미만 오름</t>
+          <t>6개월 동안 200% 이상 800% 미만 오름</t>
         </is>
       </c>
       <c r="C38" s="7" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="39" ht="32" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>손익비</t>
+          <t>6개월 상승률</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
+          <t>6개월 동안 50% 이상 200% 미만 오름</t>
         </is>
       </c>
       <c r="C39" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>손익비</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C39"/>
+  <autoFilter ref="A1:C40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Score +1 when both trendlines rise and the 1-month window is down on 6m/1y lookbacks.
Drop the 2-month window uptrend bonus.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v69</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v70</t>
         </is>
       </c>
     </row>
@@ -792,39 +792,37 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>조회 기간이 3개월 이상이고, 조회기간 2개월 조회시 상승 추세일때</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>횡보일 때</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>추세</t>
+          <t>하락 추세선 근접</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>횡보일 때</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>0</v>
+          <t>하락 추세선에 근접 했을 때</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>하락 추세선 근접</t>
+          <t>추세선 방향</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>하락 추세선에 근접 했을 때</t>
+          <t>하락 추세선 상승 추세선 모두 하락일 때</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
@@ -839,11 +837,13 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>하락 추세선 상승 추세선 모두 하락일 때</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>-1</v>
+          <t>6개월,1년 조회시 하락 추세선 상승 추세선 모두 상승이면서 1개월 조회시 하락일때</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">

</xml_diff>

<commit_message>
Award +1 on 3m+ lookbacks when trend is up/sideways and price is near the 1-month uptrend line.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v70</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v71</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>조회 기간이 3개월 이상이고, 조회기간 1개월 조회시 상승 추세일때</t>
+          <t>조회 기간이 3개월 이상이고 상승추세이거나 횡보인데 조회기간 1개월 조회시 상승추세선에 근접했을때</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Widen proximity to 1.0% of price or 0.55 ATR, whichever is larger.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v71</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v72</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1662,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>가까운 가격: 하루 변동폭의 약 절반, 또는 주가의 0.8% 중 더 큰 값.</t>
+          <t>가까운 가격: 하루 변동폭의 약 55%, 또는 주가의 1.0% 중 더 큰 값.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Evaluate 1-month trend windows on 1-hour bars when the main lookback is 3 months or more.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v72</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v73</t>
         </is>
       </c>
     </row>
@@ -644,6 +644,13 @@
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>참고: 6개월 상승률은 180일 전 종가 대비입니다. 그날이 주말·휴장이면 근처 거래일 종가를 씁니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>3개월 이상 조회에서 1개월 창(상승선·1개월 추세)은 일봉이 아니라 1개월 조회와 같은 1시간봉 30일을 씁니다.</t>
         </is>
       </c>
     </row>
@@ -775,7 +782,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>조회 기간이 3개월 이상이고 상승추세이거나 횡보인데 조회기간 1개월 조회시 상승추세선에 근접했을때</t>
+          <t>조회 기간이 3개월 이상이고 상승추세이거나 횡보인데 조회기간 1개월(1시간봉) 상승추세선에 근접했을때</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -837,7 +844,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>6개월,1년 조회시 하락 추세선 상승 추세선 모두 상승이면서 1개월 조회시 하락일때</t>
+          <t>6개월,1년 조회시 하락 추세선 상승 추세선 모두 상승이면서 1개월(1시간봉) 조회시 하락일때</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Drop the weak volume-support air-pocket penalty.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="매수 매도 기준" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v73</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v74</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -965,16 +965,18 @@
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>약한 매물대</t>
+          <t>최대 매물 (POC)</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>아래 지지 매물대가 약하고, 그 아래 다음 지지가 10% 이상 떨어져 있을 때</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>-1</v>
+          <t>현재가가 거래가 가장 많았던 가격 근처이고, 상승 추세</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
@@ -985,28 +987,28 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>현재가가 거래가 가장 많았던 가격 근처이고, 상승 추세</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>현재가가 그 가격 근처이고, 하락 추세</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>최대 매물 (POC)</t>
+          <t>밸류 하단 (VAL)</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>현재가가 그 가격 근처이고, 하락 추세</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>-1</v>
+          <t>현재가가 싼 구간 아래이고, 상승 추세</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
@@ -1017,43 +1019,43 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>현재가가 싼 구간 아래이고, 상승 추세</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>현재가가 싼 구간 아래이고, 하락 추세</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>밸류 하단 (VAL)</t>
+          <t>밸류 상단 (VAH)</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>현재가가 싼 구간 아래이고, 하락 추세</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n">
-        <v>0</v>
+          <t>현재가가 비싼 구간 위</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>밸류 상단 (VAH)</t>
+          <t>RSI</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>현재가가 비싼 구간 위</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="n">
-        <v>-1</v>
+          <t>30 이하 (너무 많이 떨어짐)</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="32" customHeight="1">
@@ -1064,13 +1066,11 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>30 이하 (너무 많이 떨어짐)</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>70 이상 (너무 많이 오름)</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="26" ht="32" customHeight="1">
@@ -1081,26 +1081,28 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>70 이상 (너무 많이 오름)</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="n">
-        <v>-1</v>
+          <t>30~70 사이</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>20일선</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>30~70 사이</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="n">
-        <v>0</v>
+          <t>현재가가 20일선보다 아래이고, 상승 추세일때</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="32" customHeight="1">
@@ -1111,13 +1113,11 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>현재가가 20일선보다 아래이고, 상승 추세일때</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>현재가가 20일선보다 아래이고, 하락 추세일때</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1">
@@ -1128,37 +1128,39 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>현재가가 20일선보다 아래이고, 하락 추세일때</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="n">
-        <v>-1</v>
+          <t>현재가가 20일선보다 아래이고, 횡보일 때</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>20일선</t>
+          <t>60일선</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>현재가가 20일선보다 아래이고, 횡보일 때</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="n">
-        <v>0</v>
+          <t>현재가가 60일(봉)선 근처일 때</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="32" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>60일선</t>
+          <t>180일선</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>현재가가 60일(봉)선 근처일 때</t>
+          <t>현재가가 장기 이평 근처일 때. 6개월 조회는 180일선, 1년 조회는 200일선</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -1170,33 +1172,33 @@
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>180일선</t>
+          <t>1개월 상승률</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>현재가가 장기 이평 근처일 때. 6개월 조회는 180일선, 1년 조회는 200일선</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>한 달 동안 30% 이상 오름</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>1개월 상승률</t>
+          <t>1개월 하락률</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 30% 이상 오름</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>-1</v>
+          <t>한 달 동안 1%이상 20%미만 하락했을시</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="32" customHeight="1">
@@ -1207,12 +1209,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 1%이상 20%미만 하락했을시</t>
+          <t>한 달 동안 20% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+2</t>
         </is>
       </c>
     </row>
@@ -1224,30 +1226,28 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 20% 이상 떨어짐</t>
+          <t>한 달 동안 40% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+3</t>
         </is>
       </c>
     </row>
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>1개월 하락률</t>
+          <t>6개월 상승률</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 40% 이상 떨어짐</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>+3</t>
-        </is>
+          <t>6개월 동안 800% 이상 오름</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>-3</v>
       </c>
     </row>
     <row r="37" ht="32" customHeight="1">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 800% 이상 오름</t>
+          <t>6개월 동안 200% 이상 800% 미만 오름</t>
         </is>
       </c>
       <c r="C37" s="7" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="38" ht="32" customHeight="1">
@@ -1273,45 +1273,30 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 200% 이상 800% 미만 오름</t>
+          <t>6개월 동안 50% 이상 200% 미만 오름</t>
         </is>
       </c>
       <c r="C38" s="7" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="39" ht="32" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>6개월 상승률</t>
+          <t>손익비</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 50% 이상 200% 미만 오름</t>
+          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
         </is>
       </c>
       <c r="C39" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="40" ht="32" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>손익비</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="n">
-        <v>-1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C40"/>
+  <autoFilter ref="A1:C39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Penalize a 4%+ opening gap on 6-month and 1-year lookbacks.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="매수 매도 기준" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v74</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v75</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1172,12 +1172,12 @@
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>1개월 상승률</t>
+          <t>갭상승</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 30% 이상 오름</t>
+          <t>6개월 이상 조회시 최근 한개봉 이전보다 4%이상 갭상승시 감점</t>
         </is>
       </c>
       <c r="C32" s="7" t="n">
@@ -1187,18 +1187,16 @@
     <row r="33" ht="32" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>1개월 하락률</t>
+          <t>1개월 상승률</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 1%이상 20%미만 하락했을시</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>한 달 동안 30% 이상 오름</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="34" ht="32" customHeight="1">
@@ -1209,12 +1207,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 20% 이상 떨어짐</t>
+          <t>한 달 동안 1%이상 20%미만 하락했을시</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+1</t>
         </is>
       </c>
     </row>
@@ -1226,28 +1224,30 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 40% 이상 떨어짐</t>
+          <t>한 달 동안 20% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+2</t>
         </is>
       </c>
     </row>
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>6개월 상승률</t>
+          <t>1개월 하락률</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 800% 이상 오름</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="n">
-        <v>-3</v>
+          <t>한 달 동안 40% 이상 떨어짐</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>+3</t>
+        </is>
       </c>
     </row>
     <row r="37" ht="32" customHeight="1">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 200% 이상 800% 미만 오름</t>
+          <t>6개월 동안 800% 이상 오름</t>
         </is>
       </c>
       <c r="C37" s="7" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="38" ht="32" customHeight="1">
@@ -1273,30 +1273,45 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 50% 이상 200% 미만 오름</t>
+          <t>6개월 동안 200% 이상 800% 미만 오름</t>
         </is>
       </c>
       <c r="C38" s="7" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="39" ht="32" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>손익비</t>
+          <t>6개월 상승률</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
+          <t>6개월 동안 50% 이상 200% 미만 오름</t>
         </is>
       </c>
       <c r="C39" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>손익비</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C39"/>
+  <autoFilter ref="A1:C40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Move the mid 1-month drop bonus from 20% to 30%.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v75</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v76</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 1%이상 20%미만 하락했을시</t>
+          <t>한 달 동안 1%이상 30%미만 하락했을시</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 20% 이상 떨어짐</t>
+          <t>한 달 동안 30% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Remove the 4% opening-gap penalty from scoring.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="매수 매도 기준" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v76</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v77</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1172,12 +1172,12 @@
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>갭상승</t>
+          <t>1개월 상승률</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>6개월 이상 조회시 최근 한개봉 이전보다 4%이상 갭상승시 감점</t>
+          <t>한 달 동안 30% 이상 오름</t>
         </is>
       </c>
       <c r="C32" s="7" t="n">
@@ -1187,16 +1187,18 @@
     <row r="33" ht="32" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>1개월 상승률</t>
+          <t>1개월 하락률</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 30% 이상 오름</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>-1</v>
+          <t>한 달 동안 1%이상 30%미만 하락했을시</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="32" customHeight="1">
@@ -1207,12 +1209,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 1%이상 30%미만 하락했을시</t>
+          <t>한 달 동안 30% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+2</t>
         </is>
       </c>
     </row>
@@ -1224,30 +1226,28 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 30% 이상 떨어짐</t>
+          <t>한 달 동안 40% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+3</t>
         </is>
       </c>
     </row>
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>1개월 하락률</t>
+          <t>6개월 상승률</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 40% 이상 떨어짐</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>+3</t>
-        </is>
+          <t>6개월 동안 800% 이상 오름</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>-3</v>
       </c>
     </row>
     <row r="37" ht="32" customHeight="1">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 800% 이상 오름</t>
+          <t>6개월 동안 200% 이상 800% 미만 오름</t>
         </is>
       </c>
       <c r="C37" s="7" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="38" ht="32" customHeight="1">
@@ -1273,45 +1273,30 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 200% 이상 800% 미만 오름</t>
+          <t>6개월 동안 50% 이상 200% 미만 오름</t>
         </is>
       </c>
       <c r="C38" s="7" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="39" ht="32" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>6개월 상승률</t>
+          <t>손익비</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 50% 이상 200% 미만 오름</t>
+          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
         </is>
       </c>
       <c r="C39" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="40" ht="32" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>손익비</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="n">
-        <v>-1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C40"/>
+  <autoFilter ref="A1:C39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Replace the 1-month uptrend-line bonus with swing low/high proximity scores.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="매수 매도 기준" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v77</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v80</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -782,39 +782,39 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>조회 기간이 3개월 이상이고 상승추세이거나 횡보인데 조회기간 1개월(1시간봉) 상승추세선에 근접했을때</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>횡보일 때</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>추세</t>
+          <t>스윙 저점 근접</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>횡보일 때</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>0</v>
+          <t>현재가가 조회 기간 스윙 저점 근처일 때</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>하락 추세선 근접</t>
+          <t>스윙 고점 근접</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>하락 추세선에 근접 했을 때</t>
+          <t>현재가가 조회 기간 스윙 고점 근처일 때</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
@@ -824,12 +824,12 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>추세선 방향</t>
+          <t>하락 추세선 근접</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>하락 추세선 상승 추세선 모두 하락일 때</t>
+          <t>하락 추세선에 근접 했을 때</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
@@ -844,24 +844,22 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>6개월,1년 조회시 하락 추세선 상승 추세선 모두 상승이면서 1개월(1시간봉) 조회시 하락일때</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>하락 추세선 상승 추세선 모두 하락일 때</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>상승 추세선 근접</t>
+          <t>추세선 방향</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>상승 추세선에 근접 했을 때</t>
+          <t>6개월,1년 조회시 하락 추세선 상승 추세선 모두 상승이면서 1개월(1시간봉) 조회시 하락일때</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -873,7 +871,7 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>상승 추세선 근접</t>
+          <t>상승 추세선 이탈</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1138,12 +1136,12 @@
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>60일선</t>
+          <t>180일선</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>현재가가 60일(봉)선 근처일 때</t>
+          <t>현재가가 장기 이평 근처일 때. 6개월 조회는 180일선, 1년 조회는 200일선</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -1155,33 +1153,33 @@
     <row r="31" ht="32" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>180일선</t>
+          <t>1개월 상승률</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>현재가가 장기 이평 근처일 때. 6개월 조회는 180일선, 1년 조회는 200일선</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
+          <t>한 달 동안 30% 이상 오름</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>1개월 상승률</t>
+          <t>1개월 하락률</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 30% 이상 오름</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="n">
-        <v>-1</v>
+          <t>한 달 동안 1%이상 30%미만 하락했을시</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1">
@@ -1192,12 +1190,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 1%이상 30%미만 하락했을시</t>
+          <t>한 달 동안 30% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+2</t>
         </is>
       </c>
     </row>
@@ -1209,30 +1207,28 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 30% 이상 떨어짐</t>
+          <t>한 달 동안 40% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+3</t>
         </is>
       </c>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>1개월 하락률</t>
+          <t>6개월 상승률</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 40% 이상 떨어짐</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>+3</t>
-        </is>
+          <t>6개월 동안 800% 이상 오름</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>-3</v>
       </c>
     </row>
     <row r="36" ht="32" customHeight="1">
@@ -1243,11 +1239,11 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 800% 이상 오름</t>
+          <t>6개월 동안 200% 이상 800% 미만 오름</t>
         </is>
       </c>
       <c r="C36" s="7" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="37" ht="32" customHeight="1">
@@ -1258,45 +1254,30 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 200% 이상 800% 미만 오름</t>
+          <t>6개월 동안 50% 이상 200% 미만 오름</t>
         </is>
       </c>
       <c r="C37" s="7" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="38" ht="32" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>6개월 상승률</t>
+          <t>손익비</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 50% 이상 200% 미만 오름</t>
+          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
         </is>
       </c>
       <c r="C38" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="39" ht="32" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>손익비</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="n">
-        <v>-1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C39"/>
+  <autoFilter ref="A1:C38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Retune 1-month and 6-month return score bands to 50/-1, 30/+1, 40/+2, 200/-1, 600/-2.
</commit_message>
<xml_diff>
--- a/규칙_점수표_v52.xlsx
+++ b/규칙_점수표_v52.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="매수 매도 기준" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기본 점수'!$A$1:$C$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'옵션 점수'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>점수 규칙 (쉬운 버전) · 지금 앱 v80</t>
+          <t>점수 규칙 (쉬운 버전) · 지금 앱 v81</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 30% 이상 오름</t>
+          <t>한 달 동안 50% 이상 오름</t>
         </is>
       </c>
       <c r="C31" s="7" t="n">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 1%이상 30%미만 하락했을시</t>
+          <t>한 달 동안 30% 이상 40% 미만 떨어짐</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 30% 이상 떨어짐</t>
+          <t>한 달 동안 40% 이상 떨어짐</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -1202,18 +1202,16 @@
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>1개월 하락률</t>
+          <t>6개월 상승률</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>한 달 동안 40% 이상 떨어짐</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>+3</t>
-        </is>
+          <t>6개월 동안 600% 이상 오름</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>-2</v>
       </c>
     </row>
     <row r="35" ht="32" customHeight="1">
@@ -1224,60 +1222,30 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 800% 이상 오름</t>
+          <t>6개월 동안 200% 이상 600% 미만 오름</t>
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>6개월 상승률</t>
+          <t>손익비</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>6개월 동안 200% 이상 800% 미만 오름</t>
+          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
         </is>
       </c>
       <c r="C36" s="7" t="n">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="37" ht="32" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>6개월 상승률</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>6개월 동안 50% 이상 200% 미만 오름</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="38" ht="32" customHeight="1">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>손익비</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>목표까지 먹을 자리보다 손절이 더 빠듯함 (1.2 미만) 그리고 점수가 이미 높은 편</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="n">
-        <v>-1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C38"/>
+  <autoFilter ref="A1:C36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>